<commit_message>
Add --dayfirst option for day/month/year files
</commit_message>
<xml_diff>
--- a/examples/output/merged.xlsx
+++ b/examples/output/merged.xlsx
@@ -682,7 +682,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2024-05-03</t>
+          <t>2024-03-05</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>2024-03-06</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -768,7 +768,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2024-06-03</t>
+          <t>2024-03-06</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2024-07-03</t>
+          <t>2024-03-07</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">

</xml_diff>